<commit_message>
- replaced capacitors that are currently not available - created gerber file and nc drill file for JLCPCB
</commit_message>
<xml_diff>
--- a/01_Altium_Project/Project Outputs for PowerTower_AdapterUltrazohm/PowerTower_AdapterUltrazohm.xlsx
+++ b/01_Altium_Project/Project Outputs for PowerTower_AdapterUltrazohm/PowerTower_AdapterUltrazohm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilflingti66489\Documents\powertower_adapter_uz\01_Altium_Project\Project Outputs for PowerTower_AdapterUltrazohm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C21B1D75-7062-4E82-83C3-DC955559A5E2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA0BBE3-8451-4D15-AE97-F36A1A71AF02}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2234,11 +2234,11 @@
       <c r="F8" s="24"/>
       <c r="G8" s="48">
         <f ca="1">TODAY()</f>
-        <v>44343</v>
+        <v>44346</v>
       </c>
       <c r="H8" s="47">
         <f ca="1">NOW()</f>
-        <v>44343.348320023149</v>
+        <v>44346.649874305556</v>
       </c>
       <c r="I8" s="28"/>
       <c r="J8" s="28"/>

</xml_diff>